<commit_message>
Ampliar estudio de mercado NPH a 3 km: 14 ofertas (5 incluidas, 9 excluidas con motivo)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WbuzTS1dj4TB6jdZmDfekN
</commit_message>
<xml_diff>
--- a/ESTUDIO_MERCADO_URBANO_BELLO_NPH_suelo.xlsx
+++ b/ESTUDIO_MERCADO_URBANO_BELLO_NPH_suelo.xlsx
@@ -32790,21 +32790,17 @@
       </c>
       <c r="F12" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">El Rosario</t>
+          <t xml:space="preserve">Altos de Niquía</t>
         </is>
       </c>
       <c r="G12" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cra 54 # 53A-23, Bello</t>
-        </is>
-      </c>
-      <c r="H12" s="94" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.3376659, -75.561891</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Urb. Altos de Niquía, cerca a la Casa de Justicia, Bello (ubicación aproximada del barrio)</t>
+        </is>
+      </c>
+      <c r="H12" s="94" t="n"/>
       <c r="I12" s="189" t="n">
-        <v>520000000</v>
+        <v>255000000</v>
       </c>
       <c r="J12" s="190">
         <f>DATOS!$C$17</f>
@@ -32815,10 +32811,10 @@
         <v/>
       </c>
       <c r="L12" s="98" t="n">
-        <v>100</v>
+        <v>99.81</v>
       </c>
       <c r="M12" s="98" t="n">
-        <v>100</v>
+        <v>99.81</v>
       </c>
       <c r="N12" s="192">
         <f>IF(A12="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A12))</f>
@@ -32846,16 +32842,16 @@
         </is>
       </c>
       <c r="T12" s="94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U12" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Casa de 100 m², 5 alcobas, 2 baños, balcón; sin administración. Publicada 01/04/2025 (reactivada 16/09/2026). A 1.611 m del objeto.</t>
+          <t xml:space="preserve">Casa de 99,81 m², 3 alcobas, 2 baños, sala-comedor, cocina semi integral, red de gas; sin administración. El portal la clasifica en piso 1 de 1 nivel. No publica coordenadas exactas: sector Altos de Niquía, vecino al objeto. Publicada 31/08/2026 (código V12194).</t>
         </is>
       </c>
       <c r="V12" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fincaraíz – Epicasa Propiedad Raíz</t>
+          <t xml:space="preserve">Fincaraíz – Arrendamientos Santa Fe</t>
         </is>
       </c>
       <c r="W12" s="94" t="inlineStr">
@@ -32865,17 +32861,17 @@
       </c>
       <c r="X12" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-el-rosario-bello/192220652</t>
+          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-bello/194185836</t>
         </is>
       </c>
       <c r="Y12" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXCLUIDA: 5 alcobas y balcón en 100 m² indican varios niveles; valor unitario atípico (≈$5,2 M/m²).</t>
+          <t xml:space="preserve">Casa NPH de 1 nivel ≤100 m² en Altos de Niquía (vecina al objeto), estrato 2. Sin coordenadas exactas; edad y estado no publicados.</t>
         </is>
       </c>
       <c r="Z12" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">SÍ</t>
         </is>
       </c>
       <c r="AA12" s="191">
@@ -32904,7 +32900,7 @@
       </c>
       <c r="C13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Casa lote</t>
+          <t xml:space="preserve">Casa</t>
         </is>
       </c>
       <c r="D13" s="94" t="inlineStr">
@@ -32919,21 +32915,21 @@
       </c>
       <c r="F13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prado – Centro de Bello</t>
+          <t xml:space="preserve">Barrio Central – La Madera</t>
         </is>
       </c>
       <c r="G13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prado Bello (sector Parque Principal), Bello</t>
+          <t xml:space="preserve">Barrio Central, Bello (San José Obrero)</t>
         </is>
       </c>
       <c r="H13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3387314, -75.5573863</t>
+          <t xml:space="preserve">6.32268, -75.5585</t>
         </is>
       </c>
       <c r="I13" s="189" t="n">
-        <v>800000000</v>
+        <v>235025000</v>
       </c>
       <c r="J13" s="190">
         <f>DATOS!$C$17</f>
@@ -32944,10 +32940,10 @@
         <v/>
       </c>
       <c r="L13" s="98" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="M13" s="98" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="N13" s="192">
         <f>IF(A13="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A13))</f>
@@ -32979,12 +32975,12 @@
       </c>
       <c r="U13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Casa lote: 2 casas (1.° y 2.° piso), ≈94 m², «para remodelar o tumbar y construir nuevamente». Publicada 09/07/2026. A 1.224 m del objeto.</t>
+          <t xml:space="preserve">Casa de 56 m², 2 alcobas, 1 baño, cocina integral, sala-comedor y zona de ropas; sin administración. No declara piso ni niveles: verificar. Publicada 05/08/2026. A 2.948 m del objeto (borde del radio de 3 km).</t>
         </is>
       </c>
       <c r="V13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fincaraíz – Bello Hogar Inmobiliaria</t>
+          <t xml:space="preserve">Ciencuadras</t>
         </is>
       </c>
       <c r="W13" s="94" t="inlineStr">
@@ -32994,17 +32990,17 @@
       </c>
       <c r="X13" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-centro-bello/193971565</t>
+          <t xml:space="preserve">https://www.ciencuadras.com/inmueble/casa-en-venta-en-san-jose-obrero-bello-3829225</t>
         </is>
       </c>
       <c r="Y13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXCLUIDA: sector Centro de Bello (otra valorización, ≈$8,5 M/m²) y son dos casas superpuestas (1.° y 2.° piso).</t>
+          <t xml:space="preserve">Casa NPH ≤100 m² dentro de 3 km, estrato 3. El anuncio no declara piso (verificar); edad y estado no publicados.</t>
         </is>
       </c>
       <c r="Z13" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">SÍ</t>
         </is>
       </c>
       <c r="AA13" s="191">
@@ -33033,7 +33029,7 @@
       </c>
       <c r="C14" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lote</t>
+          <t xml:space="preserve">Casa</t>
         </is>
       </c>
       <c r="D14" s="94" t="inlineStr">
@@ -33048,15 +33044,19 @@
       </c>
       <c r="F14" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Navarra – El Parque</t>
+          <t xml:space="preserve">El Rosario</t>
         </is>
       </c>
       <c r="G14" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autopista Norte con Calle 46, barrio El Parque, Bello (ubicación aproximada del portal)</t>
-        </is>
-      </c>
-      <c r="H14" s="94" t="n"/>
+          <t xml:space="preserve">Cra 54 # 53A-23, Bello</t>
+        </is>
+      </c>
+      <c r="H14" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3376659, -75.561891</t>
+        </is>
+      </c>
       <c r="I14" s="189" t="n">
         <v>520000000</v>
       </c>
@@ -33069,9 +33069,11 @@
         <v/>
       </c>
       <c r="L14" s="98" t="n">
-        <v>80</v>
-      </c>
-      <c r="M14" s="98" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="M14" s="98" t="n">
+        <v>100</v>
+      </c>
       <c r="N14" s="192">
         <f>IF(A14="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A14))</f>
         <v/>
@@ -33102,12 +33104,12 @@
       </c>
       <c r="U14" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lote de ≈80 m², «piso N.º 1», estrato 3, código 32643. El portal no publica coordenadas exactas (referencias a ≈1,7 km del objeto). $6,5 M/m²: probable que incluya construcción o sea valor de Centro.</t>
+          <t xml:space="preserve">Casa de 100 m², 5 alcobas, 2 baños, balcón; sin administración. Publicada 01/04/2025 (reactivada 16/09/2026). A 1.611 m del objeto.</t>
         </is>
       </c>
       <c r="V14" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metrocuadrado</t>
+          <t xml:space="preserve">Fincaraíz – Epicasa Propiedad Raíz</t>
         </is>
       </c>
       <c r="W14" s="94" t="inlineStr">
@@ -33117,12 +33119,12 @@
       </c>
       <c r="X14" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.metrocuadrado.com/inmueble/venta-lote-bello-la-navarra/2895-M6045475</t>
+          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-el-rosario-bello/192220652</t>
         </is>
       </c>
       <c r="Y14" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXCLUIDA: valor unitario atípico (≈$6,5 M/m²), sin coordenadas exactas y sin confirmar si tiene construcción.</t>
+          <t xml:space="preserve">EXCLUIDA: 5 alcobas y balcón en 100 m² indican varios niveles; valor unitario atípico (≈$5,2 M/m²).</t>
         </is>
       </c>
       <c r="Z14" s="94" t="inlineStr">
@@ -33156,7 +33158,7 @@
       </c>
       <c r="C15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lote</t>
+          <t xml:space="preserve">Casa lote</t>
         </is>
       </c>
       <c r="D15" s="94" t="inlineStr">
@@ -33171,21 +33173,21 @@
       </c>
       <c r="F15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Azulita (Niquía)</t>
+          <t xml:space="preserve">Prado – Centro de Bello</t>
         </is>
       </c>
       <c r="G15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Niquía – La Azulita, Bello</t>
+          <t xml:space="preserve">Prado Bello (sector Parque Principal), Bello</t>
         </is>
       </c>
       <c r="H15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.34284, -75.534635</t>
+          <t xml:space="preserve">6.3387314, -75.5573863</t>
         </is>
       </c>
       <c r="I15" s="189" t="n">
-        <v>160000000</v>
+        <v>800000000</v>
       </c>
       <c r="J15" s="190">
         <f>DATOS!$C$17</f>
@@ -33196,9 +33198,11 @@
         <v/>
       </c>
       <c r="L15" s="98" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="M15" s="98" t="n"/>
+        <v>94</v>
+      </c>
+      <c r="M15" s="98" t="n">
+        <v>94</v>
+      </c>
       <c r="N15" s="192">
         <f>IF(A15="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A15))</f>
         <v/>
@@ -33225,16 +33229,16 @@
         </is>
       </c>
       <c r="T15" s="94" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lote de 98,8 m², estrato 2. Publicada 04/04/2025 (≈18 meses). A 2.031 m del objeto, al oriente.</t>
+          <t xml:space="preserve">Casa lote: 2 casas (1.° y 2.° piso), ≈94 m², «para remodelar o tumbar y construir nuevamente». Publicada 09/07/2026. A 1.224 m del objeto.</t>
         </is>
       </c>
       <c r="V15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ciencuadras</t>
+          <t xml:space="preserve">Fincaraíz – Bello Hogar Inmobiliaria</t>
         </is>
       </c>
       <c r="W15" s="94" t="inlineStr">
@@ -33244,12 +33248,12 @@
       </c>
       <c r="X15" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.ciencuadras.com/inmueble/lote-en-venta-en-niquia-bello-3299412</t>
+          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-centro-bello/193971565</t>
         </is>
       </c>
       <c r="Y15" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXCLUIDA: único lote ≤100 m² encontrado, pero publicado hace más de 12 meses (vigencia) y a ≈2,0 km.</t>
+          <t xml:space="preserve">EXCLUIDA: sector Centro de Bello (otra valorización, ≈$8,5 M/m²) y son dos casas superpuestas (1.° y 2.° piso).</t>
         </is>
       </c>
       <c r="Z15" s="94" t="inlineStr">
@@ -33275,15 +33279,41 @@
       </c>
     </row>
     <row r="16" ht="57" customHeight="1" s="54">
-      <c r="A16" s="92" t="n"/>
-      <c r="B16" s="93" t="n"/>
-      <c r="C16" s="94" t="n"/>
-      <c r="D16" s="94" t="n"/>
-      <c r="E16" s="94" t="n"/>
-      <c r="F16" s="94" t="n"/>
-      <c r="G16" s="94" t="n"/>
+      <c r="A16" s="92" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lote</t>
+        </is>
+      </c>
+      <c r="D16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La Navarra – El Parque</t>
+        </is>
+      </c>
+      <c r="G16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Autopista Norte con Calle 46, barrio El Parque, Bello (ubicación aproximada del portal)</t>
+        </is>
+      </c>
       <c r="H16" s="94" t="n"/>
-      <c r="I16" s="189" t="n"/>
+      <c r="I16" s="189" t="n">
+        <v>520000000</v>
+      </c>
       <c r="J16" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33292,7 +33322,9 @@
         <f>IF(I16="","",I16*(1-J16))</f>
         <v/>
       </c>
-      <c r="L16" s="98" t="n"/>
+      <c r="L16" s="98" t="n">
+        <v>80</v>
+      </c>
       <c r="M16" s="98" t="n"/>
       <c r="N16" s="192">
         <f>IF(A16="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A16))</f>
@@ -33314,14 +33346,44 @@
         <f>IF(OR(K16="",N(M16)&lt;=0),"",K16/M16)</f>
         <v/>
       </c>
-      <c r="S16" s="94" t="n"/>
-      <c r="T16" s="94" t="n"/>
-      <c r="U16" s="94" t="n"/>
-      <c r="V16" s="94" t="n"/>
-      <c r="W16" s="94" t="n"/>
-      <c r="X16" s="100" t="n"/>
-      <c r="Y16" s="94" t="n"/>
-      <c r="Z16" s="94" t="n"/>
+      <c r="S16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T16" s="94" t="n">
+        <v>3</v>
+      </c>
+      <c r="U16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lote de ≈80 m², «piso N.º 1», estrato 3, código 32643. El portal no publica coordenadas exactas (referencias a ≈1,7 km del objeto). $6,5 M/m²: probable que incluya construcción o sea valor de Centro.</t>
+        </is>
+      </c>
+      <c r="V16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metrocuadrado</t>
+        </is>
+      </c>
+      <c r="W16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X16" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.metrocuadrado.com/inmueble/venta-lote-bello-la-navarra/2895-M6045475</t>
+        </is>
+      </c>
+      <c r="Y16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: valor unitario atípico (≈$6,5 M/m²), sin coordenadas exactas y sin confirmar si tiene construcción.</t>
+        </is>
+      </c>
+      <c r="Z16" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA16" s="191">
         <f>IF(AND(Z16="SÍ",ISNUMBER(P16)),P16,"")</f>
         <v/>
@@ -33340,15 +33402,45 @@
       </c>
     </row>
     <row r="17" ht="45.6" customHeight="1" s="54">
-      <c r="A17" s="92" t="n"/>
-      <c r="B17" s="93" t="n"/>
-      <c r="C17" s="94" t="n"/>
-      <c r="D17" s="94" t="n"/>
-      <c r="E17" s="94" t="n"/>
-      <c r="F17" s="94" t="n"/>
-      <c r="G17" s="94" t="n"/>
-      <c r="H17" s="94" t="n"/>
-      <c r="I17" s="189" t="n"/>
+      <c r="A17" s="92" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lote</t>
+        </is>
+      </c>
+      <c r="D17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La Azulita (Niquía)</t>
+        </is>
+      </c>
+      <c r="G17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Niquía – La Azulita, Bello</t>
+        </is>
+      </c>
+      <c r="H17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.34284, -75.534635</t>
+        </is>
+      </c>
+      <c r="I17" s="189" t="n">
+        <v>160000000</v>
+      </c>
       <c r="J17" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33357,7 +33449,9 @@
         <f>IF(I17="","",I17*(1-J17))</f>
         <v/>
       </c>
-      <c r="L17" s="98" t="n"/>
+      <c r="L17" s="98" t="n">
+        <v>98.8</v>
+      </c>
       <c r="M17" s="98" t="n"/>
       <c r="N17" s="192">
         <f>IF(A17="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A17))</f>
@@ -33379,14 +33473,44 @@
         <f>IF(OR(K17="",N(M17)&lt;=0),"",K17/M17)</f>
         <v/>
       </c>
-      <c r="S17" s="94" t="n"/>
-      <c r="T17" s="94" t="n"/>
-      <c r="U17" s="94" t="n"/>
-      <c r="V17" s="94" t="n"/>
-      <c r="W17" s="94" t="n"/>
-      <c r="X17" s="100" t="n"/>
-      <c r="Y17" s="94" t="n"/>
-      <c r="Z17" s="94" t="n"/>
+      <c r="S17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T17" s="94" t="n">
+        <v>2</v>
+      </c>
+      <c r="U17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lote de 98,8 m², estrato 2. Publicada 04/04/2025 (≈18 meses). A 2.031 m del objeto, al oriente.</t>
+        </is>
+      </c>
+      <c r="V17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ciencuadras</t>
+        </is>
+      </c>
+      <c r="W17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X17" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ciencuadras.com/inmueble/lote-en-venta-en-niquia-bello-3299412</t>
+        </is>
+      </c>
+      <c r="Y17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: único lote ≤100 m² encontrado, pero publicado hace más de 12 meses (vigencia) y a ≈2,0 km.</t>
+        </is>
+      </c>
+      <c r="Z17" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA17" s="191">
         <f>IF(AND(Z17="SÍ",ISNUMBER(P17)),P17,"")</f>
         <v/>
@@ -33405,15 +33529,45 @@
       </c>
     </row>
     <row r="18" ht="57" customHeight="1" s="54">
-      <c r="A18" s="92" t="n"/>
-      <c r="B18" s="93" t="n"/>
-      <c r="C18" s="94" t="n"/>
-      <c r="D18" s="94" t="n"/>
-      <c r="E18" s="94" t="n"/>
-      <c r="F18" s="94" t="n"/>
-      <c r="G18" s="94" t="n"/>
-      <c r="H18" s="94" t="n"/>
-      <c r="I18" s="189" t="n"/>
+      <c r="A18" s="92" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa</t>
+        </is>
+      </c>
+      <c r="D18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Santa Ana (Salento)</t>
+        </is>
+      </c>
+      <c r="G18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Barrio Santa Ana, Bello</t>
+        </is>
+      </c>
+      <c r="H18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.330361, -75.563075</t>
+        </is>
+      </c>
+      <c r="I18" s="189" t="n">
+        <v>235000000</v>
+      </c>
       <c r="J18" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33422,8 +33576,12 @@
         <f>IF(I18="","",I18*(1-J18))</f>
         <v/>
       </c>
-      <c r="L18" s="98" t="n"/>
-      <c r="M18" s="98" t="n"/>
+      <c r="L18" s="98" t="n">
+        <v>72</v>
+      </c>
+      <c r="M18" s="98" t="n">
+        <v>72</v>
+      </c>
       <c r="N18" s="192">
         <f>IF(A18="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A18))</f>
         <v/>
@@ -33444,14 +33602,44 @@
         <f>IF(OR(K18="",N(M18)&lt;=0),"",K18/M18)</f>
         <v/>
       </c>
-      <c r="S18" s="94" t="n"/>
-      <c r="T18" s="94" t="n"/>
-      <c r="U18" s="94" t="n"/>
-      <c r="V18" s="94" t="n"/>
-      <c r="W18" s="94" t="n"/>
-      <c r="X18" s="100" t="n"/>
-      <c r="Y18" s="94" t="n"/>
-      <c r="Z18" s="94" t="n"/>
+      <c r="S18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T18" s="94" t="n">
+        <v>3</v>
+      </c>
+      <c r="U18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa en piso 1, 72 m², 3 alcobas, 1 baño, sala, zona de ropas, red de gas. Publicada 15/08/2024 (≈25 meses). A 2.345 m del objeto.</t>
+        </is>
+      </c>
+      <c r="V18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ciencuadras</t>
+        </is>
+      </c>
+      <c r="W18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X18" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ciencuadras.com/inmueble/casa-en-venta-en-salento-bello-3068153</t>
+        </is>
+      </c>
+      <c r="Y18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: oferta publicada hace más de 12 meses (vigencia).</t>
+        </is>
+      </c>
+      <c r="Z18" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA18" s="191">
         <f>IF(AND(Z18="SÍ",ISNUMBER(P18)),P18,"")</f>
         <v/>
@@ -33470,15 +33658,45 @@
       </c>
     </row>
     <row r="19" ht="57" customHeight="1" s="54">
-      <c r="A19" s="92" t="n"/>
-      <c r="B19" s="93" t="n"/>
-      <c r="C19" s="94" t="n"/>
-      <c r="D19" s="94" t="n"/>
-      <c r="E19" s="94" t="n"/>
-      <c r="F19" s="94" t="n"/>
-      <c r="G19" s="94" t="n"/>
-      <c r="H19" s="94" t="n"/>
-      <c r="I19" s="189" t="n"/>
+      <c r="A19" s="92" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa</t>
+        </is>
+      </c>
+      <c r="D19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altos de Quitasol (Niquía)</t>
+        </is>
+      </c>
+      <c r="G19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sector Niquía, cerca a la Clínica del Norte, Bello</t>
+        </is>
+      </c>
+      <c r="H19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.34734, -75.544915</t>
+        </is>
+      </c>
+      <c r="I19" s="189" t="n">
+        <v>150000000</v>
+      </c>
       <c r="J19" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33487,8 +33705,12 @@
         <f>IF(I19="","",I19*(1-J19))</f>
         <v/>
       </c>
-      <c r="L19" s="98" t="n"/>
-      <c r="M19" s="98" t="n"/>
+      <c r="L19" s="98" t="n">
+        <v>60</v>
+      </c>
+      <c r="M19" s="98" t="n">
+        <v>60</v>
+      </c>
       <c r="N19" s="192">
         <f>IF(A19="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A19))</f>
         <v/>
@@ -33509,14 +33731,44 @@
         <f>IF(OR(K19="",N(M19)&lt;=0),"",K19/M19)</f>
         <v/>
       </c>
-      <c r="S19" s="94" t="n"/>
-      <c r="T19" s="94" t="n"/>
-      <c r="U19" s="94" t="n"/>
-      <c r="V19" s="94" t="n"/>
-      <c r="W19" s="94" t="n"/>
-      <c r="X19" s="100" t="n"/>
-      <c r="Y19" s="94" t="n"/>
-      <c r="Z19" s="94" t="n"/>
+      <c r="S19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T19" s="94" t="n">
+        <v>1</v>
+      </c>
+      <c r="U19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa bifamiliar de ≈60 m² en 1.° piso, 4 alcobas, 1 baño. Publicada 19/01/2023 (≈45 meses). A 806 m del objeto.</t>
+        </is>
+      </c>
+      <c r="V19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ciencuadras</t>
+        </is>
+      </c>
+      <c r="W19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X19" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ciencuadras.com/inmueble/casa-en-venta-en-altos-de-quitasol-bello-2574452</t>
+        </is>
+      </c>
+      <c r="Y19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: bifamiliar (derecho sobre un piso) y publicada hace más de 12 meses.</t>
+        </is>
+      </c>
+      <c r="Z19" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA19" s="191">
         <f>IF(AND(Z19="SÍ",ISNUMBER(P19)),P19,"")</f>
         <v/>
@@ -33535,15 +33787,45 @@
       </c>
     </row>
     <row r="20" ht="57" customHeight="1" s="54">
-      <c r="A20" s="92" t="n"/>
-      <c r="B20" s="93" t="n"/>
-      <c r="C20" s="94" t="n"/>
-      <c r="D20" s="94" t="n"/>
-      <c r="E20" s="94" t="n"/>
-      <c r="F20" s="94" t="n"/>
-      <c r="G20" s="94" t="n"/>
-      <c r="H20" s="94" t="n"/>
-      <c r="I20" s="189" t="n"/>
+      <c r="A20" s="92" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa</t>
+        </is>
+      </c>
+      <c r="D20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La Florida</t>
+        </is>
+      </c>
+      <c r="G20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calle 31 # 56-50, La Florida, Bello</t>
+        </is>
+      </c>
+      <c r="H20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3373933, -75.5591154</t>
+        </is>
+      </c>
+      <c r="I20" s="189" t="n">
+        <v>360000000</v>
+      </c>
       <c r="J20" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33552,8 +33834,12 @@
         <f>IF(I20="","",I20*(1-J20))</f>
         <v/>
       </c>
-      <c r="L20" s="98" t="n"/>
-      <c r="M20" s="98" t="n"/>
+      <c r="L20" s="98" t="n">
+        <v>64</v>
+      </c>
+      <c r="M20" s="98" t="n">
+        <v>64</v>
+      </c>
       <c r="N20" s="192">
         <f>IF(A20="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A20))</f>
         <v/>
@@ -33574,14 +33860,44 @@
         <f>IF(OR(K20="",N(M20)&lt;=0),"",K20/M20)</f>
         <v/>
       </c>
-      <c r="S20" s="94" t="n"/>
-      <c r="T20" s="94" t="n"/>
-      <c r="U20" s="94" t="n"/>
-      <c r="V20" s="94" t="n"/>
-      <c r="W20" s="94" t="n"/>
-      <c r="X20" s="100" t="n"/>
-      <c r="Y20" s="94" t="n"/>
-      <c r="Z20" s="94" t="n"/>
+      <c r="S20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T20" s="94" t="n">
+        <v>3</v>
+      </c>
+      <c r="U20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa unifamiliar de 64,74 m² distribuida en dos pisos por escalas, 4 alcobas, 2 baños, garaje; «piso 1 sin ascensor». Publicada 20/11/2025. A 1.449 m del objeto.</t>
+        </is>
+      </c>
+      <c r="V20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fincaraíz – Viva Inmobiliaria Asociados</t>
+        </is>
+      </c>
+      <c r="W20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X20" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-la-florida-bello/193120373</t>
+        </is>
+      </c>
+      <c r="Y20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: construcción en dos niveles; el área de lote (≈mitad del área construida) no está publicada.</t>
+        </is>
+      </c>
+      <c r="Z20" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA20" s="191">
         <f>IF(AND(Z20="SÍ",ISNUMBER(P20)),P20,"")</f>
         <v/>
@@ -33600,15 +33916,45 @@
       </c>
     </row>
     <row r="21" ht="57" customHeight="1" s="54">
-      <c r="A21" s="92" t="n"/>
-      <c r="B21" s="93" t="n"/>
-      <c r="C21" s="94" t="n"/>
-      <c r="D21" s="94" t="n"/>
-      <c r="E21" s="94" t="n"/>
-      <c r="F21" s="94" t="n"/>
-      <c r="G21" s="94" t="n"/>
-      <c r="H21" s="94" t="n"/>
-      <c r="I21" s="189" t="n"/>
+      <c r="A21" s="92" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apartamento</t>
+        </is>
+      </c>
+      <c r="D21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Barrio Nuevo (Centro)</t>
+        </is>
+      </c>
+      <c r="G21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Barrio Nuevo, Centro, Bello</t>
+        </is>
+      </c>
+      <c r="H21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3368149, -75.5596054</t>
+        </is>
+      </c>
+      <c r="I21" s="189" t="n">
+        <v>480000000</v>
+      </c>
       <c r="J21" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33618,7 +33964,9 @@
         <v/>
       </c>
       <c r="L21" s="98" t="n"/>
-      <c r="M21" s="98" t="n"/>
+      <c r="M21" s="98" t="n">
+        <v>90</v>
+      </c>
       <c r="N21" s="192">
         <f>IF(A21="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A21))</f>
         <v/>
@@ -33639,14 +33987,44 @@
         <f>IF(OR(K21="",N(M21)&lt;=0),"",K21/M21)</f>
         <v/>
       </c>
-      <c r="S21" s="94" t="n"/>
-      <c r="T21" s="94" t="n"/>
-      <c r="U21" s="94" t="n"/>
-      <c r="V21" s="94" t="n"/>
-      <c r="W21" s="94" t="n"/>
-      <c r="X21" s="100" t="n"/>
-      <c r="Y21" s="94" t="n"/>
-      <c r="Z21" s="94" t="n"/>
+      <c r="S21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T21" s="94" t="n">
+        <v>3</v>
+      </c>
+      <c r="U21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inmueble de 90 m² con terraza «del tamaño del área del apartamento»; sin administración. Publicada 22/06/2026. A 1.533 m del objeto.</t>
+        </is>
+      </c>
+      <c r="V21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fincaraíz – Casabuena Inmobiliaria</t>
+        </is>
+      </c>
+      <c r="W21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X21" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-bello/193903267</t>
+        </is>
+      </c>
+      <c r="Y21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: el propio anuncio lo describe como apartamento (derechos sobre un piso).</t>
+        </is>
+      </c>
+      <c r="Z21" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA21" s="191">
         <f>IF(AND(Z21="SÍ",ISNUMBER(P21)),P21,"")</f>
         <v/>
@@ -33665,15 +34043,41 @@
       </c>
     </row>
     <row r="22" ht="57" customHeight="1" s="54">
-      <c r="A22" s="92" t="n"/>
-      <c r="B22" s="93" t="n"/>
-      <c r="C22" s="94" t="n"/>
-      <c r="D22" s="94" t="n"/>
-      <c r="E22" s="94" t="n"/>
-      <c r="F22" s="94" t="n"/>
-      <c r="G22" s="94" t="n"/>
+      <c r="A22" s="92" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" s="93" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa</t>
+        </is>
+      </c>
+      <c r="D22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bello</t>
+        </is>
+      </c>
+      <c r="F22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Villa Occidente</t>
+        </is>
+      </c>
+      <c r="G22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Villa Occidente, cerca al Liceo Antioquia y Hospital Mental, Bello (ubicación aproximada)</t>
+        </is>
+      </c>
       <c r="H22" s="94" t="n"/>
-      <c r="I22" s="189" t="n"/>
+      <c r="I22" s="189" t="n">
+        <v>550000000</v>
+      </c>
       <c r="J22" s="190">
         <f>DATOS!$C$17</f>
         <v/>
@@ -33682,8 +34086,12 @@
         <f>IF(I22="","",I22*(1-J22))</f>
         <v/>
       </c>
-      <c r="L22" s="98" t="n"/>
-      <c r="M22" s="98" t="n"/>
+      <c r="L22" s="98" t="n">
+        <v>97</v>
+      </c>
+      <c r="M22" s="98" t="n">
+        <v>97</v>
+      </c>
       <c r="N22" s="192">
         <f>IF(A22="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A22))</f>
         <v/>
@@ -33704,14 +34112,44 @@
         <f>IF(OR(K22="",N(M22)&lt;=0),"",K22/M22)</f>
         <v/>
       </c>
-      <c r="S22" s="94" t="n"/>
-      <c r="T22" s="94" t="n"/>
-      <c r="U22" s="94" t="n"/>
-      <c r="V22" s="94" t="n"/>
-      <c r="W22" s="94" t="n"/>
-      <c r="X22" s="100" t="n"/>
-      <c r="Y22" s="94" t="n"/>
-      <c r="Z22" s="94" t="n"/>
+      <c r="S22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
+      <c r="T22" s="94" t="n">
+        <v>3</v>
+      </c>
+      <c r="U22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa de 97 m², 4 alcobas, 3 baños, parqueadero; sector Villa Occidente (≈3 km del objeto). Publicada 31/08/2026 (código V13479).</t>
+        </is>
+      </c>
+      <c r="V22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fincaraíz – Arrendamientos Santa Fe</t>
+        </is>
+      </c>
+      <c r="W22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X22" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.fincaraiz.com.co/casa-en-venta-en-bello/194185867</t>
+        </is>
+      </c>
+      <c r="Y22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXCLUIDA: valor unitario atípico (≈$5,7 M/m²), 4 alcobas y 3 baños en 97 m² indican varios niveles y queda en el borde del radio.</t>
+        </is>
+      </c>
+      <c r="Z22" s="94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO</t>
+        </is>
+      </c>
       <c r="AA22" s="191">
         <f>IF(AND(Z22="SÍ",ISNUMBER(P22)),P22,"")</f>
         <v/>
@@ -34910,7 +35348,7 @@
     <row r="58" ht="15" customHeight="1" s="54">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OBSERVACIONES DEL ESTUDIO – VALOR DE SUELO URBANO, BELLO (04/10/2026): 1) Objeto: lote urbano en 6.3484251, -75.5521303 (Niquía, Bello). Criterios de depuración: área ≤100 m²; no PH (sin administración, unidad cerrada ni conjunto); no segundo piso o superior; lote vacío o casa/casa-lote de la que se descuenta la construcción (Ross-Heidecke). 2) Fuentes consultadas: Fincaraíz (52 lotes y 160 casas de Bello), Ciencuadras (24 lotes y 27 casas) y Metrocuadrado (35 lotes y 50 casas). MercadoLibre y Properati bloquean la consulta automática y OLX no está habilitado en la red del entorno; no se revisaron. 3) Los portales solo muestran una parte de los anuncios de cada categoría; no es el universo completo. 4) De ≈370 anuncios revisados, solo 3 cumplen todos los criterios y quedan como SÍ (ofertas 1 a 3, todas casas de 1 nivel a menos de 1,5 km). Las ofertas 4 a 7 se conservan como EXCLUIDAS con su motivo. Lotes vacíos ≤100 m²: solo 2 (ofertas 6 y 7), ambos excluidos. 5) SUPUESTOS A VALIDAR (ver DEPRECIACIÓN): los anuncios no publican edad, estado ni área de lote. Se supuso área de terreno = área publicada (casa de 1 nivel), edad 30 años, vida útil 70, estado 2,5 (oferta 2: 2,0 por remodelada) y reposición $1.600.000/m². Confirmar con visita, catálogo de tipologías IGAC y consulta predial. 6) Las coordenadas son las del portal (se dejó vacía la de la oferta 6, que no publica ubicación exacta). 7) Con solo 3 ofertas incluidas el análisis del Art. 21 (mínimo 3, CV ≤ 7,5 %) es frágil: se requiere ampliar la muestra con indagación directa en campo.</t>
+          <t xml:space="preserve">OBSERVACIONES DEL ESTUDIO – VALOR DE SUELO URBANO, BELLO (04/10/2026): 1) Objeto: lote urbano en 6.3484251, -75.5521303 (Niquía, Bello). Radio de búsqueda: 3 km. Criterios de depuración: área ≤100 m²; no PH (sin administración, unidad cerrada ni conjunto); no segundo piso o superior; lote vacío o casa de un nivel de la que se descuenta la construcción (Ross-Heidecke). 2) Fuentes consultadas: Fincaraíz (52 lotes, 160 casas y 5 casas-lote de Bello), Ciencuadras (24 lotes y 27 casas) y Metrocuadrado (35 lotes y 50 casas). MercadoLibre, Properati, OLX, Mitula, Punto Propiedad y Espacio Urbano no son accesibles desde la red del entorno; no se revisaron. 3) Los portales solo muestran una parte de los anuncios de cada categoría; no es el universo completo. 4) De ≈380 anuncios revisados, 5 cumplen los criterios y quedan como SÍ (ofertas 1 a 5, casas de un nivel dentro de 3 km); las ofertas 3 y 5 no declaran el piso y deben verificarse. Las ofertas 6 a 14 se conservan como EXCLUIDAS con su motivo. Solo hay 2 lotes vacíos ≤100 m² (ofertas 8 y 9), ambos excluidos. 5) Casas de varios niveles (p. ej. 60 m² construidos en 3 pisos) no se usaron: el área de lote no está publicada y no puede suponerse igual al área construida. 6) SUPUESTOS A VALIDAR (ver DEPRECIACIÓN): los anuncios no publican edad, estado ni área de lote. Se supuso área de terreno = área publicada (casa de 1 nivel), edad 30 años, vida útil 70, estado 2,5 (oferta 2: 2,0 por remodelada) y reposición $1.600.000/m². Confirmar con visita, catálogo de tipologías IGAC y consulta predial. 7) Las coordenadas son las del portal; se dejaron vacías en las ofertas 4, 8 y 14, que no publican ubicación exacta (el portal usa un punto genérico del municipio). 8) Con 5 ofertas el análisis del Art. 21 (CV ≤ 7,5 %) es frágil: se requiere ampliar la muestra con indagación directa en campo.</t>
         </is>
       </c>
     </row>
@@ -55141,7 +55579,7 @@
       </c>
       <c r="B8" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Casa – El Rosario, Cra 54 (oferta 4, excluida)</t>
+          <t xml:space="preserve">Casa 1 nivel – Altos de Niquía (oferta 4)</t>
         </is>
       </c>
       <c r="C8" s="74" t="n">
@@ -55189,7 +55627,7 @@
         <v/>
       </c>
       <c r="O8" s="76" t="n">
-        <v>100</v>
+        <v>99.81</v>
       </c>
       <c r="P8" s="202">
         <f>IF($B8="","",MROUND(N8*O8,100))</f>
@@ -55222,17 +55660,17 @@
       </c>
       <c r="B9" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dos casas para demoler – Prado Centro (oferta 5, excluida)</t>
+          <t xml:space="preserve">Casa – Barrio Central / La Madera (oferta 5)</t>
         </is>
       </c>
       <c r="C9" s="74" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D9" s="74" t="n">
         <v>70</v>
       </c>
       <c r="E9" s="74" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F9" s="212" t="n">
         <v>1600000</v>
@@ -55270,7 +55708,7 @@
         <v/>
       </c>
       <c r="O9" s="76" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="P9" s="202">
         <f>IF($B9="","",MROUND(N9*O9,100))</f>
@@ -55298,12 +55736,26 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="74" t="n"/>
-      <c r="B10" s="70" t="n"/>
-      <c r="C10" s="74" t="n"/>
-      <c r="D10" s="74" t="n"/>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="212" t="n"/>
+      <c r="A10" s="74" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa – El Rosario, Cra 54 (oferta 6, excluida)</t>
+        </is>
+      </c>
+      <c r="C10" s="74" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="E10" s="74" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="212" t="n">
+        <v>1600000</v>
+      </c>
       <c r="G10" s="32">
         <f>IF($B10="","",MIN(C10/D10,1))</f>
         <v/>
@@ -55336,7 +55788,9 @@
         <f>IF($B10="","",IF(M10&lt;=0,0,MROUND(M10,1000)))</f>
         <v/>
       </c>
-      <c r="O10" s="76" t="n"/>
+      <c r="O10" s="76" t="n">
+        <v>100</v>
+      </c>
       <c r="P10" s="202">
         <f>IF($B10="","",MROUND(N10*O10,100))</f>
         <v/>
@@ -55345,7 +55799,11 @@
         <f>IF(AND($B10&lt;&gt;"",$A10=""),SUMPRODUCT((LEN($A$5:$A10)=0)*(LEN($B$5:$B10)&gt;0)),"")</f>
         <v/>
       </c>
-      <c r="R10" s="70" t="n"/>
+      <c r="R10" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPUESTO (edad, estado y reposición no publicados en el anuncio): validar con visita y catálogo IGAC</t>
+        </is>
+      </c>
       <c r="T10" s="25" t="n">
         <v>3</v>
       </c>
@@ -55359,12 +55817,26 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="74" t="n"/>
-      <c r="B11" s="70" t="n"/>
-      <c r="C11" s="74" t="n"/>
-      <c r="D11" s="74" t="n"/>
-      <c r="E11" s="74" t="n"/>
-      <c r="F11" s="212" t="n"/>
+      <c r="A11" s="74" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dos casas para demoler – Prado Centro (oferta 7, excluida)</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="D11" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="E11" s="74" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="212" t="n">
+        <v>1600000</v>
+      </c>
       <c r="G11" s="32">
         <f>IF($B11="","",MIN(C11/D11,1))</f>
         <v/>
@@ -55397,7 +55869,9 @@
         <f>IF($B11="","",IF(M11&lt;=0,0,MROUND(M11,1000)))</f>
         <v/>
       </c>
-      <c r="O11" s="76" t="n"/>
+      <c r="O11" s="76" t="n">
+        <v>94</v>
+      </c>
       <c r="P11" s="202">
         <f>IF($B11="","",MROUND(N11*O11,100))</f>
         <v/>
@@ -55406,7 +55880,11 @@
         <f>IF(AND($B11&lt;&gt;"",$A11=""),SUMPRODUCT((LEN($A$5:$A11)=0)*(LEN($B$5:$B11)&gt;0)),"")</f>
         <v/>
       </c>
-      <c r="R11" s="70" t="n"/>
+      <c r="R11" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPUESTO (edad, estado y reposición no publicados en el anuncio): validar con visita y catálogo IGAC</t>
+        </is>
+      </c>
       <c r="T11" s="25" t="n">
         <v>3.5</v>
       </c>
@@ -55420,12 +55898,26 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="74" t="n"/>
-      <c r="B12" s="70" t="n"/>
-      <c r="C12" s="74" t="n"/>
-      <c r="D12" s="74" t="n"/>
-      <c r="E12" s="74" t="n"/>
-      <c r="F12" s="212" t="n"/>
+      <c r="A12" s="74" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa – Santa Ana (oferta 10, excluida)</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="n">
+        <v>30</v>
+      </c>
+      <c r="D12" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="E12" s="74" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F12" s="212" t="n">
+        <v>1600000</v>
+      </c>
       <c r="G12" s="32">
         <f>IF($B12="","",MIN(C12/D12,1))</f>
         <v/>
@@ -55458,7 +55950,9 @@
         <f>IF($B12="","",IF(M12&lt;=0,0,MROUND(M12,1000)))</f>
         <v/>
       </c>
-      <c r="O12" s="76" t="n"/>
+      <c r="O12" s="76" t="n">
+        <v>72</v>
+      </c>
       <c r="P12" s="202">
         <f>IF($B12="","",MROUND(N12*O12,100))</f>
         <v/>
@@ -55467,7 +55961,11 @@
         <f>IF(AND($B12&lt;&gt;"",$A12=""),SUMPRODUCT((LEN($A$5:$A12)=0)*(LEN($B$5:$B12)&gt;0)),"")</f>
         <v/>
       </c>
-      <c r="R12" s="70" t="n"/>
+      <c r="R12" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPUESTO (edad, estado y reposición no publicados en el anuncio): validar con visita y catálogo IGAC</t>
+        </is>
+      </c>
       <c r="T12" s="25" t="n">
         <v>4</v>
       </c>
@@ -55481,12 +55979,26 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="74" t="n"/>
-      <c r="B13" s="70" t="n"/>
-      <c r="C13" s="74" t="n"/>
-      <c r="D13" s="74" t="n"/>
-      <c r="E13" s="74" t="n"/>
-      <c r="F13" s="212" t="n"/>
+      <c r="A13" s="74" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa bifamiliar – Altos de Quitasol (oferta 11, excluida)</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="n">
+        <v>30</v>
+      </c>
+      <c r="D13" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="E13" s="74" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F13" s="212" t="n">
+        <v>1600000</v>
+      </c>
       <c r="G13" s="32">
         <f>IF($B13="","",MIN(C13/D13,1))</f>
         <v/>
@@ -55519,7 +56031,9 @@
         <f>IF($B13="","",IF(M13&lt;=0,0,MROUND(M13,1000)))</f>
         <v/>
       </c>
-      <c r="O13" s="76" t="n"/>
+      <c r="O13" s="76" t="n">
+        <v>60</v>
+      </c>
       <c r="P13" s="202">
         <f>IF($B13="","",MROUND(N13*O13,100))</f>
         <v/>
@@ -55528,7 +56042,11 @@
         <f>IF(AND($B13&lt;&gt;"",$A13=""),SUMPRODUCT((LEN($A$5:$A13)=0)*(LEN($B$5:$B13)&gt;0)),"")</f>
         <v/>
       </c>
-      <c r="R13" s="70" t="n"/>
+      <c r="R13" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPUESTO (edad, estado y reposición no publicados en el anuncio): validar con visita y catálogo IGAC</t>
+        </is>
+      </c>
       <c r="T13" s="25" t="n">
         <v>4.5</v>
       </c>
@@ -55542,12 +56060,26 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="74" t="n"/>
-      <c r="B14" s="70" t="n"/>
-      <c r="C14" s="74" t="n"/>
-      <c r="D14" s="74" t="n"/>
-      <c r="E14" s="74" t="n"/>
-      <c r="F14" s="212" t="n"/>
+      <c r="A14" s="74" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa 2 niveles – La Florida (oferta 12, excluida)</t>
+        </is>
+      </c>
+      <c r="C14" s="74" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="E14" s="74" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F14" s="212" t="n">
+        <v>1600000</v>
+      </c>
       <c r="G14" s="32">
         <f>IF($B14="","",MIN(C14/D14,1))</f>
         <v/>
@@ -55580,7 +56112,9 @@
         <f>IF($B14="","",IF(M14&lt;=0,0,MROUND(M14,1000)))</f>
         <v/>
       </c>
-      <c r="O14" s="76" t="n"/>
+      <c r="O14" s="76" t="n">
+        <v>64.74</v>
+      </c>
       <c r="P14" s="202">
         <f>IF($B14="","",MROUND(N14*O14,100))</f>
         <v/>
@@ -55589,7 +56123,11 @@
         <f>IF(AND($B14&lt;&gt;"",$A14=""),SUMPRODUCT((LEN($A$5:$A14)=0)*(LEN($B$5:$B14)&gt;0)),"")</f>
         <v/>
       </c>
-      <c r="R14" s="70" t="n"/>
+      <c r="R14" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPUESTO (edad, estado y reposición no publicados en el anuncio): validar con visita y catálogo IGAC</t>
+        </is>
+      </c>
       <c r="T14" s="25" t="n">
         <v>5</v>
       </c>
@@ -55603,12 +56141,26 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="74" t="n"/>
-      <c r="B15" s="70" t="n"/>
-      <c r="C15" s="74" t="n"/>
-      <c r="D15" s="74" t="n"/>
-      <c r="E15" s="74" t="n"/>
-      <c r="F15" s="212" t="n"/>
+      <c r="A15" s="74" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa – Villa Occidente (oferta 14, excluida)</t>
+        </is>
+      </c>
+      <c r="C15" s="74" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" s="74" t="n">
+        <v>70</v>
+      </c>
+      <c r="E15" s="74" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F15" s="212" t="n">
+        <v>1600000</v>
+      </c>
       <c r="G15" s="32">
         <f>IF($B15="","",MIN(C15/D15,1))</f>
         <v/>
@@ -55641,7 +56193,9 @@
         <f>IF($B15="","",IF(M15&lt;=0,0,MROUND(M15,1000)))</f>
         <v/>
       </c>
-      <c r="O15" s="76" t="n"/>
+      <c r="O15" s="76" t="n">
+        <v>97</v>
+      </c>
       <c r="P15" s="202">
         <f>IF($B15="","",MROUND(N15*O15,100))</f>
         <v/>
@@ -55650,7 +56204,11 @@
         <f>IF(AND($B15&lt;&gt;"",$A15=""),SUMPRODUCT((LEN($A$5:$A15)=0)*(LEN($B$5:$B15)&gt;0)),"")</f>
         <v/>
       </c>
-      <c r="R15" s="70" t="n"/>
+      <c r="R15" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPUESTO (edad, estado y reposición no publicados en el anuncio): validar con visita y catálogo IGAC</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="54">
       <c r="A16" s="74" t="n"/>

</xml_diff>